<commit_message>
Update lith associated elements
</commit_message>
<xml_diff>
--- a/Codelist Excel Files and Conversion Templates to XML/USCSSoilComponents.xlsx
+++ b/Codelist Excel Files and Conversion Templates to XML/USCSSoilComponents.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="11214"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="10719"/>
   <workbookPr codeName="ThisWorkbook"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/dponti/GitHub/def/Codelist Excel Files and Conversion Templates to XML/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/dponti/Documents/GitHub/def/Codelist Excel Files and Conversion Templates to XML/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3713B3F1-49A0-5A46-980F-A9911AFFFA70}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9E8B99AE-9BC9-4243-9CD2-ADEDB7F2EC65}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="19820" yWindow="8760" windowWidth="35840" windowHeight="20900" tabRatio="500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="15360" yWindow="6320" windowWidth="35840" windowHeight="20900" tabRatio="500" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="DictionaryName" sheetId="3" r:id="rId1"/>
@@ -812,13 +812,13 @@
     <t>Particle sizes only. Silt and clay are distinguished in ASTM by their plasticity characteristics.</t>
   </si>
   <si>
-    <t>//diggs:ComponentLith/classificationCode</t>
-  </si>
-  <si>
     <t>Unified Soil Classification System Soil Component Names</t>
   </si>
   <si>
     <t>These are values defined in ASTM D2487 to define the basic components of a soil, eg. sand, silt, gravel, etc. These codes are to be used in the classificationCode property for ComponentLith objects when describing specific components wihin a soil in detail.</t>
+  </si>
+  <si>
+    <t>//diggs:classificationCode</t>
   </si>
 </sst>
 </file>
@@ -1114,6 +1114,42 @@
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="12"/>
+        <color theme="1"/>
+        <name val="Calibri"/>
+        <scheme val="minor"/>
+      </font>
+      <alignment horizontal="general" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
       <font>
         <color auto="1"/>
       </font>
@@ -1212,42 +1248,6 @@
       </font>
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
-    <dxf>
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="general" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="12"/>
-        <color theme="1"/>
-        <name val="Calibri"/>
-        <scheme val="minor"/>
-      </font>
-      <alignment horizontal="general" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
   </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleMedium7"/>
   <extLst>
@@ -1262,33 +1262,33 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="DictionaryName" displayName="DictionaryName" ref="A1:E3" totalsRowShown="0" headerRowDxfId="20" dataDxfId="19">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="DictionaryName" displayName="DictionaryName" ref="A1:E3" totalsRowShown="0" headerRowDxfId="10" dataDxfId="9">
   <autoFilter ref="A1:E3" xr:uid="{00000000-0009-0000-0100-000002000000}"/>
   <tableColumns count="5">
-    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0000-000001000000}" name="Start" dataDxfId="18"/>
-    <tableColumn id="4" xr3:uid="{00000000-0010-0000-0000-000004000000}" name="Dictionary ID" dataDxfId="17"/>
-    <tableColumn id="5" xr3:uid="{00000000-0010-0000-0000-000005000000}" name="DictionaryFile" dataDxfId="16"/>
-    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0000-000002000000}" name="DictionaryName" dataDxfId="15"/>
-    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0000-000003000000}" name="Description" dataDxfId="14"/>
+    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0000-000001000000}" name="Start" dataDxfId="8"/>
+    <tableColumn id="4" xr3:uid="{00000000-0010-0000-0000-000004000000}" name="Dictionary ID" dataDxfId="7"/>
+    <tableColumn id="5" xr3:uid="{00000000-0010-0000-0000-000005000000}" name="DictionaryFile" dataDxfId="6"/>
+    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0000-000002000000}" name="DictionaryName" dataDxfId="5"/>
+    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0000-000003000000}" name="Description" dataDxfId="4"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium9" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{00000000-000C-0000-FFFF-FFFF01000000}" name="Definitions" displayName="Definitions" ref="A1:H8" totalsRowShown="0" headerRowDxfId="13" dataDxfId="12">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{00000000-000C-0000-FFFF-FFFF01000000}" name="Definitions" displayName="Definitions" ref="A1:H8" totalsRowShown="0" headerRowDxfId="20" dataDxfId="19">
   <autoFilter ref="A1:H8" xr:uid="{00000000-0009-0000-0100-000001000000}"/>
   <tableColumns count="8">
-    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0100-000001000000}" name="Start" dataDxfId="11">
+    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0100-000001000000}" name="Start" dataDxfId="18">
       <calculatedColumnFormula>IF(ISNA(VLOOKUP(B2,AssociatedElements!B$2:B2825,1,FALSE)),"Not used","")</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="10" xr3:uid="{00000000-0010-0000-0100-00000A000000}" name="ID" dataDxfId="10"/>
-    <tableColumn id="7" xr3:uid="{00000000-0010-0000-0100-000007000000}" name="Name" dataDxfId="9"/>
-    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0100-000003000000}" name="Description" dataDxfId="8"/>
-    <tableColumn id="4" xr3:uid="{00000000-0010-0000-0100-000004000000}" name="DataType" dataDxfId="7"/>
-    <tableColumn id="5" xr3:uid="{00000000-0010-0000-0100-000005000000}" name="QuantityClass" dataDxfId="6"/>
-    <tableColumn id="6" xr3:uid="{00000000-0010-0000-0100-000006000000}" name="Authority" dataDxfId="5"/>
-    <tableColumn id="9" xr3:uid="{00000000-0010-0000-0100-000009000000}" name="Reference" dataDxfId="4"/>
+    <tableColumn id="10" xr3:uid="{00000000-0010-0000-0100-00000A000000}" name="ID" dataDxfId="17"/>
+    <tableColumn id="7" xr3:uid="{00000000-0010-0000-0100-000007000000}" name="Name" dataDxfId="16"/>
+    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0100-000003000000}" name="Description" dataDxfId="15"/>
+    <tableColumn id="4" xr3:uid="{00000000-0010-0000-0100-000004000000}" name="DataType" dataDxfId="14"/>
+    <tableColumn id="5" xr3:uid="{00000000-0010-0000-0100-000005000000}" name="QuantityClass" dataDxfId="13"/>
+    <tableColumn id="6" xr3:uid="{00000000-0010-0000-0100-000006000000}" name="Authority" dataDxfId="12"/>
+    <tableColumn id="9" xr3:uid="{00000000-0010-0000-0100-000009000000}" name="Reference" dataDxfId="11"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium9" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -1636,10 +1636,10 @@
         <v>233</v>
       </c>
       <c r="D3" s="2" t="s">
+        <v>258</v>
+      </c>
+      <c r="E3" s="2" t="s">
         <v>259</v>
-      </c>
-      <c r="E3" s="2" t="s">
-        <v>260</v>
       </c>
     </row>
   </sheetData>
@@ -1904,7 +1904,7 @@
         <v>235</v>
       </c>
       <c r="C2" s="3" t="s">
-        <v>258</v>
+        <v>260</v>
       </c>
     </row>
     <row r="3" spans="1:4" ht="17" x14ac:dyDescent="0.2">
@@ -1916,7 +1916,7 @@
         <v>239</v>
       </c>
       <c r="C3" s="3" t="s">
-        <v>258</v>
+        <v>260</v>
       </c>
     </row>
     <row r="4" spans="1:4" ht="17" x14ac:dyDescent="0.2">
@@ -1928,7 +1928,7 @@
         <v>242</v>
       </c>
       <c r="C4" s="3" t="s">
-        <v>258</v>
+        <v>260</v>
       </c>
     </row>
     <row r="5" spans="1:4" ht="17" x14ac:dyDescent="0.2">
@@ -1940,7 +1940,7 @@
         <v>244</v>
       </c>
       <c r="C5" s="3" t="s">
-        <v>258</v>
+        <v>260</v>
       </c>
     </row>
     <row r="6" spans="1:4" ht="17" x14ac:dyDescent="0.2">
@@ -1952,7 +1952,7 @@
         <v>247</v>
       </c>
       <c r="C6" s="3" t="s">
-        <v>258</v>
+        <v>260</v>
       </c>
     </row>
     <row r="7" spans="1:4" ht="17" x14ac:dyDescent="0.2">
@@ -1964,7 +1964,7 @@
         <v>251</v>
       </c>
       <c r="C7" s="3" t="s">
-        <v>258</v>
+        <v>260</v>
       </c>
     </row>
     <row r="8" spans="1:4" ht="17" x14ac:dyDescent="0.2">
@@ -1976,7 +1976,7 @@
         <v>254</v>
       </c>
       <c r="C8" s="3" t="s">
-        <v>258</v>
+        <v>260</v>
       </c>
     </row>
   </sheetData>

</xml_diff>